<commit_message>
Sync planning SharePoint : S30
</commit_message>
<xml_diff>
--- a/Plannings 2026 S30.xlsx
+++ b/Plannings 2026 S30.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{DEC38800-D319-4A77-B909-3492472F2FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{720229C2-D327-4A92-9E29-0DF6CB07D80D}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{DEC38800-D319-4A77-B909-3492472F2FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B04291E-C539-4312-8485-B355F432F5BE}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="105">
   <si>
     <t>Planning des salariés du 20/07/2026 au 26/07/2026</t>
   </si>
@@ -87,9 +87,6 @@
     <t>11:00/18:30</t>
   </si>
   <si>
-    <t>11:45/18:30</t>
-  </si>
-  <si>
     <t>11:45/18:05</t>
   </si>
   <si>
@@ -334,6 +331,12 @@
   </si>
   <si>
     <t>STAGE // P100</t>
+  </si>
+  <si>
+    <t>11:45/16:00</t>
+  </si>
+  <si>
+    <t>19:00/21:10</t>
   </si>
 </sst>
 </file>
@@ -4843,6 +4846,270 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="50" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B048E98-A7D9-46B1-976F-92FE88EBCDD6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="609600" y="3438525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="51" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{742707EF-246F-4C73-A13F-73CEFDA06D44}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1219200" y="3438525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="52" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C99C2462-1588-4E01-9FF1-3341968B465F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="3438525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="53" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A21A894-A1B1-4F8D-A334-6DCD6518CDA4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1828800" y="3819525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="54" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F46C3C0C-4835-49DD-B8A6-023B69C991B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2438400" y="3438525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>123825</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="97" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6BEFDE2-5D2E-4CD7-95F7-58C5C72C46C8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3048000" y="3438525"/>
+          <a:ext cx="123825" cy="123825"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -5245,19 +5512,19 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -5305,7 +5572,7 @@
         <v>13</v>
       </c>
       <c r="B6" s="27" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" s="28"/>
       <c r="D6" s="28"/>
@@ -5344,67 +5611,71 @@
       <c r="A9" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="18"/>
-      <c r="H9" s="19"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="41"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>22</v>
+      </c>
       <c r="G10" s="3"/>
-      <c r="H10" s="22"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="41"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="2" t="s">
+        <v>15</v>
+      </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="22"/>
+      <c r="H11" s="3"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="35"/>
-      <c r="B12" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="G12" s="20"/>
-      <c r="H12" s="21"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
     </row>
     <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="28"/>
@@ -5416,20 +5687,20 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" s="13" t="s">
         <v>26</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>27</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="22" t="s">
@@ -5439,34 +5710,34 @@
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="36"/>
       <c r="B15" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="13" t="s">
         <v>30</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>31</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="36"/>
       <c r="B16" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="3"/>
@@ -5475,14 +5746,14 @@
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="36"/>
       <c r="B17" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="3"/>
@@ -5491,7 +5762,7 @@
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="36"/>
       <c r="B18" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -5505,12 +5776,12 @@
     <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="35"/>
       <c r="B19" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C19" s="20"/>
       <c r="D19" s="20"/>
       <c r="E19" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F19" s="25"/>
       <c r="G19" s="20"/>
@@ -5518,22 +5789,22 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="23" t="s">
-        <v>40</v>
-      </c>
       <c r="C20" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F20" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G20" s="18"/>
       <c r="H20" s="19"/>
@@ -5541,19 +5812,19 @@
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="36"/>
       <c r="B21" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="E21" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" s="15" t="s">
         <v>41</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="E21" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="F21" s="15" t="s">
-        <v>42</v>
       </c>
       <c r="G21" s="3"/>
       <c r="H21" s="22"/>
@@ -5561,19 +5832,19 @@
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" s="36"/>
       <c r="B22" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F22" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G22" s="3"/>
       <c r="H22" s="22"/>
@@ -5581,19 +5852,19 @@
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" s="36"/>
       <c r="B23" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G23" s="3"/>
       <c r="H23" s="22"/>
@@ -5601,19 +5872,19 @@
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" s="36"/>
       <c r="B24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G24" s="3"/>
       <c r="H24" s="22"/>
@@ -5621,19 +5892,19 @@
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" s="36"/>
       <c r="B25" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G25" s="3"/>
       <c r="H25" s="22"/>
@@ -5641,19 +5912,19 @@
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" s="36"/>
       <c r="B26" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G26" s="3"/>
       <c r="H26" s="22"/>
@@ -5661,19 +5932,19 @@
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" s="36"/>
       <c r="B27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G27" s="3"/>
       <c r="H27" s="22"/>
@@ -5681,17 +5952,17 @@
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" s="36"/>
       <c r="B28" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F28" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G28" s="3"/>
       <c r="H28" s="22"/>
@@ -5699,17 +5970,17 @@
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" s="36"/>
       <c r="B29" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C29" s="15"/>
       <c r="D29" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G29" s="3"/>
       <c r="H29" s="22"/>
@@ -5717,11 +5988,11 @@
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="36"/>
       <c r="B30" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" s="15"/>
       <c r="D30" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E30" s="15"/>
       <c r="F30" s="15"/>
@@ -5731,11 +6002,11 @@
     <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="35"/>
       <c r="B31" s="24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C31" s="24"/>
       <c r="D31" s="24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E31" s="24"/>
       <c r="F31" s="24"/>
@@ -5744,14 +6015,14 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>15</v>
@@ -5767,20 +6038,20 @@
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="36"/>
       <c r="B33" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="F33" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="H33" s="22"/>
     </row>
@@ -5801,7 +6072,7 @@
       <c r="B35" s="20"/>
       <c r="C35" s="20"/>
       <c r="D35" s="20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E35" s="20"/>
       <c r="F35" s="20"/>
@@ -5810,7 +6081,7 @@
     </row>
     <row r="36" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B36" s="27"/>
       <c r="C36" s="28"/>
@@ -5822,7 +6093,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="34" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B37" s="18"/>
       <c r="C37" s="18"/>
@@ -5841,7 +6112,7 @@
       <c r="B38" s="20"/>
       <c r="C38" s="20"/>
       <c r="D38" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>16</v>
@@ -5852,7 +6123,7 @@
     </row>
     <row r="39" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B39" s="27"/>
       <c r="C39" s="28"/>
@@ -5864,22 +6135,22 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" s="34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G40" s="18"/>
       <c r="H40" s="19"/>
@@ -5887,19 +6158,19 @@
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" s="36"/>
       <c r="B41" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C41" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="15" t="s">
-        <v>42</v>
-      </c>
       <c r="D41" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E41" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E41" s="15" t="s">
-        <v>42</v>
-      </c>
       <c r="F41" s="15" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G41" s="3"/>
       <c r="H41" s="22"/>
@@ -5907,19 +6178,19 @@
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" s="36"/>
       <c r="B42" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F42" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G42" s="3"/>
       <c r="H42" s="22"/>
@@ -5927,19 +6198,19 @@
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" s="36"/>
       <c r="B43" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D43" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E43" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G43" s="3"/>
       <c r="H43" s="22"/>
@@ -5947,19 +6218,19 @@
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" s="36"/>
       <c r="B44" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F44" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G44" s="3"/>
       <c r="H44" s="22"/>
@@ -5967,19 +6238,19 @@
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" s="36"/>
       <c r="B45" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E45" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F45" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G45" s="3"/>
       <c r="H45" s="22"/>
@@ -5987,19 +6258,19 @@
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" s="36"/>
       <c r="B46" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G46" s="3"/>
       <c r="H46" s="22"/>
@@ -6007,19 +6278,19 @@
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" s="36"/>
       <c r="B47" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E47" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G47" s="3"/>
       <c r="H47" s="22"/>
@@ -6028,14 +6299,14 @@
       <c r="A48" s="36"/>
       <c r="B48" s="15"/>
       <c r="C48" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D48" s="15"/>
       <c r="E48" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F48" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G48" s="3"/>
       <c r="H48" s="22"/>
@@ -6044,14 +6315,14 @@
       <c r="A49" s="36"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D49" s="15"/>
       <c r="E49" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F49" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G49" s="3"/>
       <c r="H49" s="22"/>
@@ -6060,11 +6331,11 @@
       <c r="A50" s="36"/>
       <c r="B50" s="15"/>
       <c r="C50" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D50" s="15"/>
       <c r="E50" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F50" s="15"/>
       <c r="G50" s="3"/>
@@ -6074,11 +6345,11 @@
       <c r="A51" s="36"/>
       <c r="B51" s="15"/>
       <c r="C51" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D51" s="15"/>
       <c r="E51" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F51" s="15"/>
       <c r="G51" s="3"/>
@@ -6090,7 +6361,7 @@
       <c r="C52" s="15"/>
       <c r="D52" s="15"/>
       <c r="E52" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F52" s="15"/>
       <c r="G52" s="3"/>
@@ -6102,7 +6373,7 @@
       <c r="C53" s="24"/>
       <c r="D53" s="24"/>
       <c r="E53" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F53" s="24"/>
       <c r="G53" s="20"/>
@@ -6110,7 +6381,7 @@
     </row>
     <row r="54" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B54" s="30"/>
       <c r="C54" s="31"/>
@@ -6122,7 +6393,7 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" s="34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B55" s="18"/>
       <c r="C55" s="18" t="s">
@@ -6140,10 +6411,10 @@
       <c r="A56" s="35"/>
       <c r="B56" s="20"/>
       <c r="C56" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D56" s="20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E56" s="20"/>
       <c r="F56" s="20"/>
@@ -6152,15 +6423,15 @@
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" s="34" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B57" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C57" s="18"/>
       <c r="D57" s="18"/>
       <c r="E57" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F57" s="18" t="s">
         <v>15</v>
@@ -6171,15 +6442,15 @@
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" s="36"/>
       <c r="B58" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="3"/>
       <c r="E58" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="22"/>
@@ -6187,12 +6458,12 @@
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" s="36"/>
       <c r="B59" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="3"/>
       <c r="E59" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -6201,12 +6472,12 @@
     <row r="60" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="35"/>
       <c r="B60" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C60" s="20"/>
       <c r="D60" s="20"/>
       <c r="E60" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F60" s="20"/>
       <c r="G60" s="20"/>
@@ -6214,7 +6485,7 @@
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" s="34" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B61" s="18"/>
       <c r="C61" s="18"/>
@@ -6236,15 +6507,15 @@
       <c r="E62" s="20"/>
       <c r="F62" s="20"/>
       <c r="G62" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="H62" s="21" t="s">
         <v>72</v>
-      </c>
-      <c r="H62" s="21" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="63" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B63" s="27"/>
       <c r="C63" s="28"/>
@@ -6256,7 +6527,7 @@
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" s="34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B64" s="18" t="s">
         <v>15</v>
@@ -6279,26 +6550,26 @@
     <row r="65" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="35"/>
       <c r="B65" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C65" s="20" t="s">
         <v>77</v>
-      </c>
-      <c r="C65" s="20" t="s">
-        <v>78</v>
       </c>
       <c r="D65" s="20"/>
       <c r="E65" s="20"/>
       <c r="F65" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="G65" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="G65" s="20" t="s">
-        <v>80</v>
-      </c>
       <c r="H65" s="21" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B66" s="30"/>
       <c r="C66" s="31"/>
@@ -6310,7 +6581,7 @@
     </row>
     <row r="67" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B67" s="27"/>
       <c r="C67" s="28"/>
@@ -6322,7 +6593,7 @@
     </row>
     <row r="68" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B68" s="27"/>
       <c r="C68" s="28"/>
@@ -6334,7 +6605,7 @@
     </row>
     <row r="69" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B69" s="27"/>
       <c r="C69" s="28"/>
@@ -6399,7 +6670,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C4" s="39"/>
       <c r="D4" s="39"/>
@@ -6407,7 +6678,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="40" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C5" s="40"/>
       <c r="D5" s="40"/>
@@ -6418,16 +6689,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -6534,7 +6805,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B13" s="8">
         <v>0</v>
@@ -6551,7 +6822,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B14" s="8">
         <v>0</v>
@@ -6568,7 +6839,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B15" s="8">
         <v>0</v>
@@ -6585,7 +6856,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B16" s="8">
         <v>0</v>
@@ -6602,7 +6873,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B17" s="8">
         <v>0</v>
@@ -6619,7 +6890,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B18" s="8">
         <v>0</v>
@@ -6636,7 +6907,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B19" s="8">
         <v>0</v>
@@ -6653,7 +6924,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B20" s="8">
         <v>0</v>
@@ -6670,7 +6941,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B21" s="8">
         <v>0</v>
@@ -6687,7 +6958,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" s="8">
         <v>0</v>
@@ -6704,7 +6975,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B23" s="8">
         <v>0</v>
@@ -6721,7 +6992,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B24" s="8">
         <v>0</v>
@@ -6738,7 +7009,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B25" s="8">
         <v>0</v>
@@ -6755,7 +7026,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B26" s="8">
         <v>0</v>
@@ -6772,7 +7043,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B27" s="8">
         <v>0</v>
@@ -6789,7 +7060,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B28" s="8">
         <v>0</v>
@@ -6806,7 +7077,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B29" s="8">
         <v>0</v>
@@ -6823,7 +7094,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B30" s="8">
         <v>0</v>
@@ -6840,7 +7111,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B31" s="8">
         <v>0</v>
@@ -6857,7 +7128,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B32" s="8">
         <v>0</v>
@@ -6874,7 +7145,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B33" s="8">
         <v>0</v>
@@ -6924,40 +7195,40 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>92</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>96</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>98</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>